<commit_message>
Add company role skill extraction pipeline
</commit_message>
<xml_diff>
--- a/data/company_roles/company_roles.xlsx
+++ b/data/company_roles/company_roles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mala/Documents/AI_engineer/jobmatch-ai/data/company_roles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAFCBD05-6B40-0745-9241-819F7DB17F0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5C306B2-2398-B14F-83F5-AD936CEABD62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16660" xr2:uid="{1257E9B8-7CD0-4247-865F-0A2697F6C5B7}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{1257E9B8-7CD0-4247-865F-0A2697F6C5B7}"/>
   </bookViews>
   <sheets>
     <sheet name="company_roles" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
   <si>
     <t>company</t>
   </si>
@@ -34,88 +34,115 @@
     <t>required_skill</t>
   </si>
   <si>
-    <t>experience_level</t>
-  </si>
-  <si>
     <t>department</t>
   </si>
   <si>
-    <t>TechNova</t>
-  </si>
-  <si>
-    <t>AI Engineer</t>
-  </si>
-  <si>
-    <t>"Develop and deploy AI systems using machine learning and NLP"</t>
-  </si>
-  <si>
-    <t>"Python;Machine Learning;NLP;PyTorch;LLM"</t>
-  </si>
-  <si>
-    <t>Mid</t>
-  </si>
-  <si>
-    <t>AI</t>
-  </si>
-  <si>
-    <t>Data Scientist</t>
-  </si>
-  <si>
-    <t>"Analyze data and build predictive models"</t>
-  </si>
-  <si>
-    <t>"Python;SQL;Statistics;Machine Learning;Pandas"</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>Backend Engineer</t>
-  </si>
-  <si>
-    <t>"Build and maintain backend services and APIs"</t>
-  </si>
-  <si>
-    <t>"Python;SQL;PostgreSQL;REST API;Docker"</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>Admin</t>
-  </si>
-  <si>
-    <t>"Manage administrative tasks, documentation, scheduling, and office operations"</t>
-  </si>
-  <si>
-    <t>"Microsoft Office;Documentation;Communication;Data Entry;Organization"</t>
-  </si>
-  <si>
-    <t>Junior</t>
-  </si>
-  <si>
-    <t>Administration</t>
-  </si>
-  <si>
-    <t>HR</t>
-  </si>
-  <si>
-    <t>"Manage recruitment, employee relations, HR administration, and talent development"</t>
-  </si>
-  <si>
-    <t>"Recruitment;Communication;HRIS;Employee Relations;Microsoft Office"</t>
+    <t>Mekari</t>
+  </si>
+  <si>
+    <t>AI and Data Specialist</t>
+  </si>
+  <si>
+    <t>The AI/Data Builder is an AI-native Builder who owns AI, ML, LLM, data, and non-deterministic system quality. This role expects to stay close to users and ships end-to-end, user-accessible AI/data products, features, modules, workflows, services, and decision-support capabilities. What sets this role apart is deeper accountability for the quality of probabilistic behavior, data quality, model behavior, evaluation systems, AI trust, guardrails, and continuous improvement. The mission: build, ship, measure, and improve AI/data capabilities that are useful, safe, trusted, measurable, and valuable for users. User &amp; product alignment. Stay close to workflows, feedback, and production behavior to define what "good vs. unacceptable" AI behavior looks like for the use case.
+Build &amp; ship. Develop AI services, ML models, LLM workflows, RAG systems, data pipelines, and model integrations as real product capabilities (not just experiments).
+Configure &amp; construct. Own prompts, retrieval logic, model configs, orchestration flows, and data transformations.
+Validate quality. Test behavior through eval sets, golden datasets, scenario/adversarial tests, regression evals, and human review.
+Manage risk. Handle grounding, hallucination, bias, privacy, latency, cost, and drift concerns.
+Release responsibly. Ship with guardrails, fallbacks, monitoring, and human-in-the-loop controls.
+Iterate. Continuously improve prompts, models, and pipelines based on real usage data.
+Cross-functional collaboration. Partner with Platform Builders (deployment, agent tuning) and Product Builders (user value, trust boundaries, release readiness).</t>
+  </si>
+  <si>
+    <t>Junior Payroll Specialist</t>
+  </si>
+  <si>
+    <t>Collect and validate employee time and attendance data. Calculate and process employee salaries, wages, bonuses, and commissions. Review and verify accuracy of payroll data, including hours worked, deductions, and taxes. Ensure compliance with applicable laws and regulations related to payroll, including tax withholding and reporting. Reconcile payroll transactions and resolve discrepancies. Generate payroll reports, including earnings statements, tax filings, and deductions summaries. Prepare and submit payroll tax returns and ensure compliance with tax laws and regulations. Stay updated on changes in payroll regulations and employment tax laws. Maintain accurate and up-to-date employee payroll records, including earnings, deductions, and taxes. Ensure data confidentiality and security in handling sensitive employee information. Collaborate with Client’s HR, Finance, and other departments to resolve payroll-related issues. Assist clients with payroll inquiries, including pay discrepancies, deductions, and tax-related matters. Identify opportunities for process improvements to enhance efficiency and accuracy of payroll operations. Work closely with the payroll team to implement new systems or tools to streamline processes.</t>
+  </si>
+  <si>
+    <t>Bachelor's degree in management, HR, or a related field (preferred). Proven experience as a payroll specialist or in a similar role. Strong knowledge of payroll practices, employment tax laws, and regulations. Proficiency in using payroll software or HRIS (Human Resources Information System), understanding Talenta is a plus. Excellent numerical and analytical skills with a keen eye for detail. Advanced proficiency in MS Excel or other spreadsheet software. Ability to handle confidential information with discretion. Strong communication and interpersonal skills. Organizational and time management skills to meet deadlines and manage multiple tasks. Problem-solving abilities and a proactive approach to resolving issues.</t>
+  </si>
+  <si>
+    <t>Coordinate with Account Manager, Customer Support, and other commercial stakeholders by clarifying the customer’s complaint. Provide technical support and win-win solution to customers for any issues that arise with the use of our products. Validate all issues being escalated. Coordinate with Product and Engineering Team to resolve product problems.</t>
+  </si>
+  <si>
+    <t>Technical Support</t>
+  </si>
+  <si>
+    <t>Candidate must possess at least a Bachelor's Degree Information System, Logistics Management, or equivalent. Fresh graduates are welcome to apply. Have basic knowledge in Logistic, Accounting Information System and E-Commerce ecosystem. Have work experience, esp. in e-commerce field will be a plus point. Familiar with MySQL will be a plus point. Proficient in English (both written and spoken). Good analytical and problem-solving skills.</t>
+  </si>
+  <si>
+    <t>SEO Associate</t>
+  </si>
+  <si>
+    <t>Create and implement comprehensive SEO Content strategies to improve search engine rankings, AI citation and drive organic traffic. Conduct thorough keyword research to identify relevant keywords and optimize content accordingly. Develop original, high-quality, &amp; engaging content (e.g., blog posts, articles) that is optimized for search engines and resonates with our target audience. Optimize articles/blog content to improve user engagement, EEAT, and rank in SERP. Monitor Blog performance and analyze content metrics to identify areas for improvement and optimize existing content. Conduct competitor analysis to stay ahead of industry trends and identify opportunities for differentiation. Work closely with the SEO Specialist &amp; outreach team to ensure content aligns with overall marketing goals and brand messaging. Collaborate with other writers and stakeholders to brainstorm ideas and refine content strategies.</t>
+  </si>
+  <si>
+    <t>At least 2 years experience in optimize SEO campaign, as a content specialist or SEO writer, or similar role. A strong understanding &amp; practical knowledge of SEO principles with AI search optimization (e.g AIO, AI Mode, LLMs) and best practices. Familiarity with SEO tools (e.g., Google Analytics, Google Search Console, SEMrush, Ahrefs, Looker Studio). Ability to create original, high-quality content by human for humans. Excellent written and verbal communication skills in Bahasa Indonesia and English. Strong research skills and the ability to write about diverse topics. Highly organized and detail-oriented. A passion for learning and staying up-to-date with the latest SEO trends. Experience with content management systems (CMS) especially Wordpress.</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Solution Engineering</t>
+  </si>
+  <si>
+    <t>The Solution Engineer is responsible for working with customers to understand their business needs and then designing, developing, and implementing custom solutions using no-code tools. The ideal candidate will have a strong understanding of software engineering principles and a passion for helping customers solve their problems. Plan: Translate business requirements into structured development plans. Develop: Write clean, efficient code to build scalable applications. Test: Create and execute automated tests to ensure application reliability. Deploy: Manage smooth rollouts of new features to production environments. Maintain: Monitor and troubleshoot any incoming bugs.</t>
+  </si>
+  <si>
+    <t>Educational background in Information Technology or Computer Science. Minimum 1 year of experience ad developer or software engineer. Have a good understanding of Javascript and CSS. Understand how to use REST API. Understand Database &amp; SQL. Strong aptitude to learn new technologies. Excellent communication and problem-solving skills. Ability to work independently and as part of a team.</t>
+  </si>
+  <si>
+    <t>Information Technology</t>
+  </si>
+  <si>
+    <t>Risk Management Specialist</t>
+  </si>
+  <si>
+    <t>Own and drive Mekari’s Enterprise Risk Management (ERM) framework end-to-end. Build and operationalize AI-powered risk management solutions by integrating LLMs with enterprise data sources and business workflows. Enable proactive risk engagement across all business units to strengthen enterprise-wide mitigation. Lead the development and continuous enhancement of the Risk Register, ensuring accurate risk identification, parameters, and scoring. Influence stakeholders and drive effective execution of risk treatment strategies across the organization. Deliver structured, actionable risk reports to senior leadership and executive stakeholders. Provide risk-based insights for internal audit planning, vendor assessments, and new product evaluations. Lead risk awareness campaigns, training programs, and communication initiatives company-wide.
+Maintain compliance readiness for ISO 27001, SOC 2, and other relevant frameworks.</t>
+  </si>
+  <si>
+    <t>3+ years of experience in risk management, preferably in SaaS or technology companies.
+Strong stakeholder management, critical thinking, and reporting capabilities. Strong understanding of internal controls, SOP governance, risk assessment, and audit follow-up processes. Excellent coordination, communication, interviewing, and influencing skills. Highly detail-oriented, assertive, and comfortable managing multiple priorities in a dynamic environment. Experience in tech, digital, or fast-paced cross-functional environments is an advantage.</t>
+  </si>
+  <si>
+    <t>Project Manager</t>
+  </si>
+  <si>
+    <t>Legal</t>
+  </si>
+  <si>
+    <t>Assist clients to set up and configure ERP modules (Finance, Inventory, Procurement, and Manufacturing/Production) according to clients' business requirements. Provide product training to users across relevant ERP modules. Provide consultancy to clients on best practices for business process automation and ERP adoption. Maintain account portfolio to ensure activation progress, system usage, and transaction activity across modules. Support and provide solutions to clients' issues, including cross-module and integration-related concerns. Gather client's business process requirements and coordinate implementation into the system. Coordinate with the developer/product team for bug testing and feedback on new ERP features. Regularly report to the manager on client's needs, adoption progress, and potential problems. Collaborate with cross-functional teams to ensure smooth end-to-end client onboarding.</t>
+  </si>
+  <si>
+    <t>Candidate must possess at least a Bachelor's Degree in Accounting, Information Systems, Business, or equivalent. Have experiences with project management, consultation and setup ERP systems before.
+Required skills: understanding of business processes (Finance, Inventory, Procurement, and/or Manufacturing). Prior exposure to ERP systems (SAP, Oracle, Odoo, or similar) is a plus. Proficient with corporate productivity and web presentation tools (Microsoft &amp; Gsuite). Excellent written and verbal communication skills. Good analytical and problem-solving skills, with the ability to translate business processes into system configuration. Fluent in English, writing and verbal. Comfortable with numbers, data, and meeting clients. Fast learner and independent, able to grasp multiple ERP modules. Good interpersonal and teamwork skills. Able to work under pressure and manage multiple client implementations simultaneously.</t>
+  </si>
+  <si>
+    <t>IT Auditor Lead</t>
+  </si>
+  <si>
+    <t>Maintain the quarterly IT internal audit plan, ensuring alignment with key risks and organizational priorities. Lead end-to-end IT audit engagements, from planning, fieldwork, to reporting. Identify and assess IT-related risks, including cybersecurity, data privacy, operational technology risks, and emerging tech risks. Evaluate the effectiveness of IT controls across applications, infrastructure, cybersecurity, cloud environments, and data governance. Review system configurations, access controls, change management, and IT operations for potential risks and control gaps. Conduct annual audits for compliance with ISO 27001 and other relevant standards or regulations, as well as special audits (e.g., investigations, security incidents, and ad hoc assignments). Drive and monitor the implementation of IT audit recommendations across relevant teams (Engineering, Product, InfoSec, IT Ops). Develop and maintain audit reports, issue logs, dashboards, and management updates on IT control health. Provide early warning indicators on emerging IT risks, system vulnerabilities, or deviations from expected controls. Support awareness initiatives related to IT governance, cybersecurity, and internal controls.</t>
+  </si>
+  <si>
+    <t>3-6 years of experience in IT Audit, IT Risk, Cybersecurity, or Technology Assurance. Strong understanding of IT general controls (ITGC), application controls, cloud environments, cybersecurity frameworks, and technology risk assessment. Familiarity with standards such as ISO 27001, SOC 2, NIST, COBIT, or similar frameworks. Strong technical foundation with familiarity in SQL, JavaScript, and Python for data analysis or system review. Relevant certifications such as CISA, CRISC, ISO 27001 Lead Auditor/Implementer are a strong plus. Strong communication, coordination, interviewing, and issue-challenging skills when dealing with technical teams. Highly detail-oriented, analytical, and comfortable managing multiple concurrent audit or review activities.</t>
+  </si>
+  <si>
+    <t>Senior QA Engineer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing estimations and prioritisations within sprints. Reviewing of test artifacts such as test cases, testrail reports, automation scripts, reported bugs on different environments and/or RFCs (if any). Setting in collaboration with EM/HOE and tracking quality metrics. Raising the quality bar by applying the best quality practices and testing techniques. Regular 1:1s with direct reports and their leader (EM or HOE). Pushing for automation skill sets within the team and automation first testing approach. Hands-on with 1 or more features. Participating in scrum events and tribe level OKR discussions. Setting squad specific OKRs driven through tribe OKRs </t>
+  </si>
+  <si>
+    <t>Automation Mastery: Deep expertise in modern automation tools (e.g., Selenium, Playwright, Cypress, or Appium) and languages (Python, Java, or JavaScript). Cloud &amp; Infrastructure: Experience testing microservices architectures hosted on AWS, Alicloud, or GCP. Familiarity with Docker and Kubernetes is a major plus. CI/CD Integration: Proven track record of integrating automated suites into pipelines like GitHub Actions, GitLab CI, or Jenkins. API Testing: Strong command of RESTful API testing and performance/load testing tools (e.g., JMeter, Locust, or k6). Knowledgeable in SQL (MySQL/PostgreSQL). Passionate as a problem solver. Proactive, vigilant, responsible, and collaborative</t>
+  </si>
+  <si>
+    <t>2 - 3+ years in full-stack engineering or applied software development using AI/data use cases. Experience with AI, ML, LLM, RAG, data, analytics, and intelligent product systems. Proficiency in prompt, context, retrieval, model, orchestration, and data-system design.
+Experience with data pipelines, data quality, freshness, lineage, completeness, and correctness. Demonstrated ability with evaluation design, golden datasets, regression evals, scenario tests, and human review. Working knowledge of grounding, hallucination control, refusal behavior, guardrails, safety, and trust.
+Experience monitoring for drift, quality degradation, latency, cost, user feedback, and production behavior. Track record shipping AI/data-powered products, features, modules, workflows, services, or decision-support capabilities. Preferred Traits, Experience collaborating with Platform Builders on agentic build workflows, especially agent tuning, evaluation, and improvement. Comfort defining risk tolerances and behavior standards for non-deterministic systems (i.e., systems where output varies based on models, prompts, retrieval, data, context, or user input, and can't be verified by exact-output tests alone). Mindset, A builder who takes deep ownership of AI/data behavior quality — someone who treats evaluation, monitoring, and continuous improvement as core parts of shipping, not afterthoughts, and who partners naturally with Product and Platform counterparts (this role isn't research-only, model-only, or analytics-only — it's about shipping real AI/data-powered capability and managing its quality in production).</t>
   </si>
   <si>
     <t>Human Resource</t>
-  </si>
-  <si>
-    <t>Finance</t>
-  </si>
-  <si>
-    <t>"Manage financial records, budgeting, reporting, and financial analysis"</t>
-  </si>
-  <si>
-    <t>"Accounting;Financial Analysis;Excel;Budgeting;Financial Reporting"</t>
   </si>
 </sst>
 </file>
@@ -599,8 +626,17 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1" shrinkToFit="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -976,147 +1012,184 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EA33047-0A32-FD4B-A5CB-39C9C626DF53}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="63.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="388" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
+      <c r="B2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="3" spans="1:5" ht="170" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="102" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
+    <row r="5" spans="1:5" ht="187" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="D5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="6" spans="1:5" ht="102" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="204" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="221" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
         <v>17</v>
       </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
+    <row r="9" spans="1:5" ht="187" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" t="s">
         <v>21</v>
       </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" t="s">
-        <v>29</v>
+    <row r="10" spans="1:5" ht="170" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>